<commit_message>
feat/fix: add Bomb class and misc. fixes
</commit_message>
<xml_diff>
--- a/Bonus/Levels/levels_list.xlsx
+++ b/Bonus/Levels/levels_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Bonus\Levels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A2039FD-1696-496C-B3A7-F82C758AC58B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B311062-FBED-4959-A2EA-8A15A18948B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
   <si>
     <t>ID</t>
   </si>
@@ -201,6 +201,30 @@
 T?T.T.T.T?T.TTT.T.T?T?T
 T.T....+...?..T.?....+T
 TTTTTTTTTTTTTTTTTTTTTTT</t>
+  </si>
+  <si>
+    <t>Koyuki and Bombs 6-7</t>
+  </si>
+  <si>
+    <t>Hmm, maybe those rocks need a little destroying…</t>
+  </si>
+  <si>
+    <t>15 15
+~~~~~~~~~~~~~~~
+~...RRRRRR....~
+~.L..R.RRR..+.~
+~..._RRRRRR...~
+~....R.RRRR...~
+~..!.RRRRRR...~
+~....RRRRRR._.~
+~..+.RRRRRR...~
+~....RRRRRR...~
+~._.R..RRRR...~
+~...RRRRRRR...~
+~......RRRR...~
+~.!.RRRRRRR._.~
+~.....RRR.....~
+~~~~~~~~~~~~~~~</t>
   </si>
 </sst>
 </file>
@@ -546,7 +570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.06640625" style="1"/>
@@ -687,6 +711,23 @@
         <v>1</v>
       </c>
     </row>
+    <row r="8" spans="1:6" ht="228" x14ac:dyDescent="0.45">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: Ice implementation & Flamethrower animations (WIP)
</commit_message>
<xml_diff>
--- a/Bonus/Levels/levels_list.xlsx
+++ b/Bonus/Levels/levels_list.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Bonus\Levels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github Repositories\cs11-project-jugemu-jugemu\Bonus\Levels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B311062-FBED-4959-A2EA-8A15A18948B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63F23453-F748-4D95-8919-8E0734B19D5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
   <si>
     <t>ID</t>
   </si>
@@ -225,6 +225,37 @@
 ~.!.RRRRRRR._.~
 ~.....RRR.....~
 ~~~~~~~~~~~~~~~</t>
+  </si>
+  <si>
+    <t>Skipping Ice</t>
+  </si>
+  <si>
+    <t>This ice is too slippery, too fast!</t>
+  </si>
+  <si>
+    <t>6 7
+TTTTTTT
+T...~+T
+T.L.~TT
+T...#.T
+T.....T
+TTTTTTT</t>
+  </si>
+  <si>
+    <t>Ice Age</t>
+  </si>
+  <si>
+    <t>Booga Booga</t>
+  </si>
+  <si>
+    <t>7 11
+T...T+T...T
+T...T~T...T
+TTTTT~TTTTT
+T.........T
+T.#..L..R.T
+T.........T
+TTTTTTTTTTT</t>
   </si>
 </sst>
 </file>
@@ -570,18 +601,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.06640625" style="1"/>
-    <col min="2" max="2" width="27.59765625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="45.265625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="28.53125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="77.796875" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.06640625" style="1"/>
+    <col min="1" max="1" width="9" style="1"/>
+    <col min="2" max="2" width="27.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="45.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="77.85546875" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.65" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -601,7 +632,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -619,7 +650,7 @@
       </c>
       <c r="F2" s="5"/>
     </row>
-    <row r="3" spans="1:6" ht="228" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" ht="240" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -637,7 +668,7 @@
       </c>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:6" ht="256.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:6" ht="270" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -655,7 +686,7 @@
       </c>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" ht="165" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -673,7 +704,7 @@
       </c>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" ht="370.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" ht="390" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -691,7 +722,7 @@
       </c>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="1:6" ht="342" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6" ht="360" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -711,7 +742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="228" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6" ht="240" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -726,6 +757,40 @@
       </c>
       <c r="E8" s="1" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="120" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: new tile beehive and mechanic bee
</commit_message>
<xml_diff>
--- a/Bonus/Levels/levels_list.xlsx
+++ b/Bonus/Levels/levels_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Bonus\Levels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B311062-FBED-4959-A2EA-8A15A18948B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E958122E-27CE-4710-8E48-2652A7A339D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
   <si>
     <t>ID</t>
   </si>
@@ -225,6 +225,23 @@
 ~.!.RRRRRRR._.~
 ~.....RRR.....~
 ~~~~~~~~~~~~~~~</t>
+  </si>
+  <si>
+    <t>Buzzer Beater</t>
+  </si>
+  <si>
+    <t>It stings!</t>
+  </si>
+  <si>
+    <t>8 30
+......RR.......&amp;......&amp;R......
+......RR.......&amp;......&amp;R......
+......RR..+....&amp;......&amp;R......
+......RR.......&amp;......&amp;R...!..
+.....+RR.......&amp;......&amp;R......
+......RR.......&amp;......&amp;R......
+.+....RR.......&amp;..L...&amp;R......
+......RR.......&amp;......&amp;R......</t>
   </si>
 </sst>
 </file>
@@ -570,7 +587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.06640625" style="1"/>
@@ -728,6 +745,23 @@
         <v>29</v>
       </c>
     </row>
+    <row r="9" spans="1:6" ht="128.25" x14ac:dyDescent="0.45">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: add Log feature and tester level
</commit_message>
<xml_diff>
--- a/Bonus/Levels/levels_list.xlsx
+++ b/Bonus/Levels/levels_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Bonus\Levels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E958122E-27CE-4710-8E48-2652A7A339D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2352DBC4-3FE5-4BE9-A74C-D9A3445CDCFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
   <si>
     <t>ID</t>
   </si>
@@ -242,6 +242,45 @@
 ......RR.......&amp;......&amp;R......
 .+....RR.......&amp;..L...&amp;R......
 ......RR.......&amp;......&amp;R......</t>
+  </si>
+  <si>
+    <t>The Cold Never Bothered Me Anyway</t>
+  </si>
+  <si>
+    <t>Just a Test</t>
+  </si>
+  <si>
+    <t>10 10
+......~...
+.T..o...0L
+.T.o..~...
+.T....~~~~
+TT........
+T...0.o..T
+..........
+..........
+.~._...x..
+.+........</t>
+  </si>
+  <si>
+    <t>So Close yet So Far</t>
+  </si>
+  <si>
+    <t>That axe must be so useful</t>
+  </si>
+  <si>
+    <t>11 20
+.............RT.....
+.............RT.....
+..L..........RT.....
+............~~T..+..
+..o.........~.T.....
+....o.......~.T.....
+............~.T.....
+....o.......~~T.....
+..o..........RT.....
+.......*.....RT.....
+.............RT.....</t>
   </si>
 </sst>
 </file>
@@ -587,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.06640625" style="1"/>
@@ -762,6 +801,40 @@
         <v>32</v>
       </c>
     </row>
+    <row r="10" spans="1:6" ht="156.75" x14ac:dyDescent="0.45">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="171" x14ac:dyDescent="0.45">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: bomb functionality, add levels
</commit_message>
<xml_diff>
--- a/Bonus/Levels/levels_list.xlsx
+++ b/Bonus/Levels/levels_list.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github Repositories\cs11-project-jugemu-jugemu\Bonus\Levels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Bonus\Levels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B57CFED5-8441-4A4E-9E3D-E35BAFAAF699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CECFF588-E59E-44C2-814B-AAD6C2747166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="51">
   <si>
     <t>ID</t>
   </si>
@@ -281,12 +281,6 @@
     <t>Just a Test</t>
   </si>
   <si>
-    <t>So Close yet So Far</t>
-  </si>
-  <si>
-    <t>That axe must be so useful</t>
-  </si>
-  <si>
     <t>11 20
 .............RT.....
 .............RT.....
@@ -312,6 +306,78 @@
 ..........
 .~._...x..
 .+........</t>
+  </si>
+  <si>
+    <t>So Close Yet So Far</t>
+  </si>
+  <si>
+    <t>Bridges are built to be burnt</t>
+  </si>
+  <si>
+    <t>Into The Beehive</t>
+  </si>
+  <si>
+    <t>You should've turned back when you go the chance.</t>
+  </si>
+  <si>
+    <t>19 30
+....T..T..........+....RRRRRRR
+....T..TTTTTTTTTTTTTTTTTRRRRRR
+..+.T..&amp;....+?...T.....TRRRRRR
+....TTTTTT.T.T.T.T.T.T?TRRRRRR
+....T..T!T.?.._..x.T+..TRRRRRR
+T.TTT..T.T.T.T.TTTTT.T.TRRRRR+
+..T._..T+T&amp;T+.+?+T&amp;..T.T.RRRRR
+..T....T.T.TTT.T.T.T.T.T.RRRRR
+..T....T.......T.T..&amp;..T..RRRR
+..TTTTTT.T.T.TTT?T.T.T.T..RRRR
+...TTTTTx.&amp;..T+T.T.?.T.T...RRR
+TTTT..TT.T.T?T.T.T.T.T.T....RR
+.....TTT?..!...T..+..T.TTT.+..
+.x..~TTT.T.T.T.TTTTTTT.T.TTT..
+..?...TT..&amp;..T.T.T+..&amp;.TTT.T..
+..L...TT.T.T.T.TTT.T.T&amp;T..?T..
+......TT!..?..+..T.T..!T...T..
+......TTTTTTTTTTTTTToTTTTTTT..
+..+....x....ooooo...o.........</t>
+  </si>
+  <si>
+    <t>How's a big boom?</t>
+  </si>
+  <si>
+    <t>29 29
+......RRRRRRRRRRRRRRRRR......
+.+...RRRRRRRRRRRRRRRRRRR...+.
+....RRRRRRRRRRRRRRRRRRRRR....
+...RRRRRRRRRRRRRRRRRRRRRRR...
+..RRRRRRRRRRRRRRRRRRRRRRRRR..
+.RRRRRRRRRRRRRRRRRRRRRRRRRRR.
+RRRRRRRRRRRRRR.RRRRRRRRRRRRRR
+RRRRRRRRRRRRR...RRRRRRRRRRRRR
+RRRRRRRRRRRRT.!..RRRRRRRRRRRR
+RRRRRRRRRRR.T.!...RRRRRRRRRRR
+RRRRRRRRRR..T......RRRRRRRRRR
+RRRRRRRRR...T.......RRRRRRRRR
+RRRRRRRR....TTTTTTTTTRRRRRRRR
+RRRRRRR.....T.x.T.....RRRRRRR
+RRRRRR..!!..TxLxT..!!..RRRRRR
+RRRRRRR.....T.x.T.....RRRRRRR
+RRRRRRRRTTTTTTTTT....RRRRRRRR
+RRRRRRRRR.......T...RRRRRRRRR
+RRRRRRRRRR......T..RRRRRRRRRR
+RRRRRRRRRRR...!.T.RRRRRRRRRRR
+RRRRRRRRRRRR..!.TRRRRRRRRRRRR
+RRRRRRRRRRRRR...RRRRRRRRRRRRR
+RRRRRRRRRRRRRR.RRRRRRRRRRRRRR
+.RRRRRRRRRRRRRRRRRRRRRRRRRRR.
+..RRRRRRRRRRRRRRRRRRRRRRRRR..
+...RRRRRRRRRRRRRRRRRRRRRRR...
+....RRRRRRRRRRRRRRRRRRRRR....
+.+...RRRRRRRRRRRRRRRRRRR...+.
+......RRRRRRRRRRRRRRRRR......</t>
+  </si>
+  <si>
+    <t>Blast Processing</t>
   </si>
 </sst>
 </file>
@@ -360,7 +426,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -376,9 +442,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -660,18 +723,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
-    <col min="2" max="2" width="27.5703125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="45.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="28.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="77.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27.59765625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="45.265625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28.59765625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="77.86328125" style="1" customWidth="1"/>
     <col min="6" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="14.65" x14ac:dyDescent="0.5">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -691,7 +754,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -709,7 +772,7 @@
       </c>
       <c r="F2" s="5"/>
     </row>
-    <row r="3" spans="1:6" ht="240" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="228" x14ac:dyDescent="0.45">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -727,7 +790,7 @@
       </c>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:6" ht="270" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="256.5" x14ac:dyDescent="0.45">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -745,7 +808,7 @@
       </c>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6" ht="165" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -763,7 +826,7 @@
       </c>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" ht="390" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="370.5" x14ac:dyDescent="0.45">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -781,7 +844,7 @@
       </c>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="1:6" ht="360" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="342" x14ac:dyDescent="0.45">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -801,7 +864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="240" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="228" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -818,58 +881,58 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="135" x14ac:dyDescent="0.25">
-      <c r="A9" s="6">
+    <row r="9" spans="1:6" ht="128.25" x14ac:dyDescent="0.45">
+      <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="6" t="s">
+      <c r="D9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="165" x14ac:dyDescent="0.25">
-      <c r="A10" s="6">
+    <row r="10" spans="1:6" ht="156.75" x14ac:dyDescent="0.45">
+      <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E10" s="6" t="s">
+      <c r="D10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="171" x14ac:dyDescent="0.45">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="180" x14ac:dyDescent="0.25">
-      <c r="A11" s="6">
-        <v>10</v>
-      </c>
-      <c r="B11" s="6" t="s">
+      <c r="D11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:6" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -886,7 +949,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="120" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="114" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -901,6 +964,43 @@
       </c>
       <c r="E13" s="1" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="285" x14ac:dyDescent="0.45">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="409.5" x14ac:dyDescent="0.45">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add folder system to excel
</commit_message>
<xml_diff>
--- a/Bonus/Levels/levels_list.xlsx
+++ b/Bonus/Levels/levels_list.xlsx
@@ -5,15 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Bonus\Levels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\cs11-project-si-legends\Bonus\Levels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CECFF588-E59E-44C2-814B-AAD6C2747166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0B640E2-67E3-455A-8A08-9E23A2ADB044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="45" yWindow="750" windowWidth="28710" windowHeight="14685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Folders" sheetId="2" r:id="rId1"/>
+    <sheet name="1" sheetId="1" r:id="rId2"/>
+    <sheet name="2" sheetId="3" r:id="rId3"/>
+    <sheet name="3" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="55">
   <si>
     <t>ID</t>
   </si>
@@ -378,6 +381,18 @@
   </si>
   <si>
     <t>Blast Processing</t>
+  </si>
+  <si>
+    <t>Testing 1</t>
+  </si>
+  <si>
+    <t>Testing 2</t>
+  </si>
+  <si>
+    <t>Testing 3</t>
+  </si>
+  <si>
+    <t>Lorem ipsum dolor sit amet, consectetur adipiscing elit.</t>
   </si>
 </sst>
 </file>
@@ -426,7 +441,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -442,6 +457,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -722,19 +740,79 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1E384E5-DA51-499D-8241-92ECB4AE2D20}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="6"/>
+    <col min="2" max="2" width="31.85546875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="77.5703125" style="6" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="6">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="6">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="6">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F15"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
-    <col min="2" max="2" width="27.59765625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="45.265625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="28.59765625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="77.86328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="45.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="77.85546875" style="1" customWidth="1"/>
     <col min="6" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.65" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -754,7 +832,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -772,7 +850,7 @@
       </c>
       <c r="F2" s="5"/>
     </row>
-    <row r="3" spans="1:6" ht="228" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" ht="240" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -790,7 +868,7 @@
       </c>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:6" ht="256.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:6" ht="270" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -808,7 +886,7 @@
       </c>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" ht="165" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -826,7 +904,7 @@
       </c>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" ht="370.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" ht="390" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -844,7 +922,7 @@
       </c>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="1:6" ht="342" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6" ht="360" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -864,7 +942,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="228" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6" ht="240" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -881,7 +959,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -898,7 +976,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:6" ht="165" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -915,7 +993,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="171" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:6" ht="180" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -932,7 +1010,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -949,7 +1027,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="114" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -966,7 +1044,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="285" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:6" ht="300" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -986,7 +1064,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1007,4 +1085,578 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66F63D6C-32C3-41F1-9B37-CC4CAED619C5}">
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9" style="1"/>
+    <col min="2" max="2" width="27.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="45.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="77.85546875" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="5"/>
+    </row>
+    <row r="3" spans="1:6" ht="240" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="5"/>
+    </row>
+    <row r="4" spans="1:6" ht="270" x14ac:dyDescent="0.25">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="5"/>
+    </row>
+    <row r="5" spans="1:6" ht="165" x14ac:dyDescent="0.25">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="5"/>
+    </row>
+    <row r="6" spans="1:6" ht="390" x14ac:dyDescent="0.25">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="5"/>
+    </row>
+    <row r="7" spans="1:6" ht="360" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="240" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="135" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="165" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="180" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="120" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="300" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1407AC4E-D895-4AE8-B12F-9065761963AC}">
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9" style="1"/>
+    <col min="2" max="2" width="27.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="45.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="77.85546875" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="5"/>
+    </row>
+    <row r="3" spans="1:6" ht="240" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="5"/>
+    </row>
+    <row r="4" spans="1:6" ht="270" x14ac:dyDescent="0.25">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="5"/>
+    </row>
+    <row r="5" spans="1:6" ht="165" x14ac:dyDescent="0.25">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="5"/>
+    </row>
+    <row r="6" spans="1:6" ht="390" x14ac:dyDescent="0.25">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="5"/>
+    </row>
+    <row r="7" spans="1:6" ht="360" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="240" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="135" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="165" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="180" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="120" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="300" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor/feat: unify utils and restructure metadata to add bee row
</commit_message>
<xml_diff>
--- a/Bonus/Levels/levels_list.xlsx
+++ b/Bonus/Levels/levels_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Bonus\Levels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD5BDA0F-F30D-48B6-9C6E-D5DE1084B4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C088D0CD-2AF4-4B46-8ED8-AC1117490446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Folders" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="63">
   <si>
     <t>ID</t>
   </si>
@@ -399,6 +399,73 @@
   </si>
   <si>
     <t>NOI.ph Horizons</t>
+  </si>
+  <si>
+    <t>29 29
+...~..RRRRRRRRTT#RRRRRR......
+.+...RRRRoRToRRRRRoRRRoR...+.
+.._.#RRRR#TTRRRRoRRRRRRRR....
+~..RRR#RRTTRRoRRR#RRRRRRRR.~.
+..RRRoRTRRoRRRR#RRRRRRRRRRR..
+.RooRRRTRRRRRRoRRRRRTRRRRRoR.
+RRoRoRRRRRRRRR##RRRRRRRRRRRRo
+RRRRRRRRTR#RTRRRRRooRRRRRRRTT
+RR#TTRRRRR#RRRRRRRRRRR#T#RRRT
+RRRRoRoRoRRRRR.#oTT#RRTRRRRTR
+RoRRRRRR#RRRR...oRTRRRRRRRR#R
+RoTTo#RRRRRR.T..!R#Ro#RRRRRRT
+RRRRTRRRR#R!.TT..!RoRRoTRRRR#
+R#RTRRRoTR!..TxTTT.RRRR#TRRRR
+RRRRoRRRR...TxLxT...oRRRRRRRR
+RRRRRRRRRR.TTTxT_.!RTRRRR##RR
+RRRRRRRooRT...TT.!TRRRRRRR#RR
+#RRRRR#RRRRR!..T.RRRRRRoRRT#T
+RRRR#RRRRRTTo!..RRRRRRRRRRRTR
+o#RTRRTRoRRooR.RRoRoRRRRRRRR#
+ooR#oR#RRRRRRRoRRRRRTRRRRRRRR
+RRRRRRRRRoRRRo#RRRR#RR#RRRT#R
+ooRTRRRRTTRTTRR#RTRoRRT#R#R#R
+.RR#RRT#RR#RR#TRRoRRoRRRRRR#.
+..RRRRRoRRRTRRToRR#ToRRRoRo..
+...RTRRoRRoRR#TRR#RRRRRRRR..~
+~...RRRooRToR##RTRRRRRR#R....
+.+...RRoRRRRooR#RRRRRRRR...+.
+..._..R#RRRRRRRTRoRoRRR......</t>
+  </si>
+  <si>
+    <t>Bee</t>
+  </si>
+  <si>
+    <t>Beelieve</t>
+  </si>
+  <si>
+    <t>There's so many of them!</t>
+  </si>
+  <si>
+    <t>3 500</t>
+  </si>
+  <si>
+    <t>20 20
+....................
+...........+........
+....................
+....................
+....+...............
+....................
+....................
+................+...
++........&amp;..........
+........&amp;L&amp;.......+.
+.........&amp;..........
+....................
+.................+..
+....................
+....................
+....................
+...+........+.......
+....................
+....................
+....................</t>
   </si>
 </sst>
 </file>
@@ -447,7 +514,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -466,6 +533,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -807,7 +877,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
@@ -818,7 +888,7 @@
     <col min="6" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.65" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:7" ht="14.65" x14ac:dyDescent="0.5">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -837,8 +907,11 @@
       <c r="F1" s="3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="G1" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -856,7 +929,7 @@
       </c>
       <c r="F2" s="5"/>
     </row>
-    <row r="3" spans="1:6" ht="228" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" ht="228" x14ac:dyDescent="0.45">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -874,7 +947,7 @@
       </c>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:6" ht="256.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" ht="256.5" x14ac:dyDescent="0.45">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -892,7 +965,7 @@
       </c>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -910,7 +983,7 @@
       </c>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" ht="370.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="370.5" x14ac:dyDescent="0.45">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -928,7 +1001,7 @@
       </c>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="1:6" ht="342" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" ht="342" x14ac:dyDescent="0.45">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -948,7 +1021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="228" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" ht="228" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -965,7 +1038,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" ht="128.25" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -982,7 +1055,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -999,7 +1072,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="171" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" ht="171" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1016,7 +1089,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1033,7 +1106,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="114" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7" ht="114" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1050,7 +1123,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="285" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" ht="285" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1070,7 +1143,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1084,7 +1157,27 @@
         <v>6</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>49</v>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="299.25" x14ac:dyDescent="0.45">
+      <c r="A16" s="1">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1095,7 +1188,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66F63D6C-32C3-41F1-9B37-CC4CAED619C5}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
@@ -1106,7 +1199,7 @@
     <col min="6" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.65" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:7" ht="14.65" x14ac:dyDescent="0.5">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1125,8 +1218,11 @@
       <c r="F1" s="3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="G1" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1144,7 +1240,7 @@
       </c>
       <c r="F2" s="5"/>
     </row>
-    <row r="3" spans="1:6" ht="228" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" ht="228" x14ac:dyDescent="0.45">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1162,7 +1258,7 @@
       </c>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:6" ht="256.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" ht="256.5" x14ac:dyDescent="0.45">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -1180,7 +1276,7 @@
       </c>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -1198,7 +1294,7 @@
       </c>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" ht="370.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="370.5" x14ac:dyDescent="0.45">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -1216,7 +1312,7 @@
       </c>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="1:6" ht="342" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" ht="342" x14ac:dyDescent="0.45">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -1236,7 +1332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="228" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" ht="228" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1253,7 +1349,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" ht="128.25" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1270,7 +1366,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1287,7 +1383,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="171" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" ht="171" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1304,7 +1400,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1321,7 +1417,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="114" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7" ht="114" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1338,7 +1434,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="285" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" ht="285" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1358,7 +1454,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1377,12 +1473,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1407AC4E-D895-4AE8-B12F-9065761963AC}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
@@ -1393,7 +1490,7 @@
     <col min="6" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.65" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:7" ht="14.65" x14ac:dyDescent="0.5">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1412,8 +1509,11 @@
       <c r="F1" s="3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="G1" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1431,7 +1531,7 @@
       </c>
       <c r="F2" s="5"/>
     </row>
-    <row r="3" spans="1:6" ht="228" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" ht="228" x14ac:dyDescent="0.45">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1449,7 +1549,7 @@
       </c>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:6" ht="256.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" ht="256.5" x14ac:dyDescent="0.45">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -1467,7 +1567,7 @@
       </c>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -1485,7 +1585,7 @@
       </c>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" ht="370.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="370.5" x14ac:dyDescent="0.45">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -1503,7 +1603,7 @@
       </c>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="1:6" ht="342" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" ht="342" x14ac:dyDescent="0.45">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -1523,7 +1623,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="228" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" ht="228" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1540,7 +1640,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" ht="128.25" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1557,7 +1657,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1574,7 +1674,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="171" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" ht="171" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1591,7 +1691,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1608,7 +1708,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="114" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7" ht="114" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1625,7 +1725,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="285" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" ht="285" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1645,7 +1745,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
chore: integrate Miguel's fixes
</commit_message>
<xml_diff>
--- a/Bonus/Levels/levels_list.xlsx
+++ b/Bonus/Levels/levels_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Bonus\Levels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C088D0CD-2AF4-4B46-8ED8-AC1117490446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E717F97-468D-4DBD-B0A3-56BB001708F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Folders" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: fix central imports
</commit_message>
<xml_diff>
--- a/Bonus/Levels/levels_list.xlsx
+++ b/Bonus/Levels/levels_list.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Bonus\Levels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A13FEA1F-77B9-4369-866D-18B59ECC0551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53EA744B-7DBF-46D8-BDE6-A4C707D9282E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Folders" sheetId="2" r:id="rId1"/>
     <sheet name="1" sheetId="1" r:id="rId2"/>
     <sheet name="2" sheetId="3" r:id="rId3"/>
     <sheet name="3" sheetId="4" r:id="rId4"/>
+    <sheet name="4" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="93">
   <si>
     <t>ID</t>
   </si>
@@ -535,12 +536,289 @@
 ........!...............RRRRR.......RRRRR....R.R.RRRRRRRRRRRRRRRRRRRRR
 _........_...............RRRRRRR.RRRRRRR...!.......R..R...RRRRRRRRRRRR</t>
   </si>
+  <si>
+    <t>Ice Test</t>
+  </si>
+  <si>
+    <t>28 11
+~~~~~~~~~~~
+~~~~~~~~~~~
+~#~TTTTT~#~
+~#TT.o.TT~#
+#TT..#..TT#
+.T.....~~T~
+TT..T.T~.TT
+T.x.T+T...T
+T...T~T.x.T
+TTTTT~TTTTT
+#~........T
+T..#...R..#
+T...~~~...T
+T#...T....T
+TT..~~~..TT
+.TT.....TT.
+..T..~..T..
+.#TT...TT..
+...T...T.#.
+~~.TT.TT.~.
+.~..T#T..__
+.#~....~~#.
+..~..L.~...
+.~~.....#..
+#~..R.R._..
+.~.RR~RR.~.
+_..RR+RR...</t>
+  </si>
+  <si>
+    <t>At the Crossroads</t>
+  </si>
+  <si>
+    <t>This island is fairly large...</t>
+  </si>
+  <si>
+    <t>3 7</t>
+  </si>
+  <si>
+    <t>50 50
+~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~RRRRRRRR~~~~~~~~
+~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~RRRRRRRR~~~~~~~~~
+~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~RRRo+RRRR~~~~~~~~~
+~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~RRRooRRRR~~~~~~~~~~
+~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~RRRooRRRR~~~~~~~~~~~
+~~~~~~~~~~~~~~~~~~~~~~~~~~~~~RRRooRRRR~~~~~~~~~~~~
+~~~~~~~~~~~~~~~~~~~~~~~~~~~RRRRooRRRR~~~~~~~~~~~~~
+~~~~~~~~~~~~~~~~~~~~~~~~~.RRRRooRRRR~~~~~~~~~~~~~~
+~~~~~~~~~~~~~~~~~~~~....RRRRRooRRRRR~~~~~~~~~~~~~~
+~~~~~~~~~~~~~~~~~..*..RRRRRoooRRRR~~~~~~~~~~~~~~~~
+~~~~~~~~~~~~~~~~...RRRRRRoooRRRRR..~~~~~~~~~~~~~~~
+~~~~~~~~~~~~~~..RRRRRRRRooRRRRR......~~~~~~~~~~~~~
+~~~~~~~~~~~~~RRRRRRRRooooRRRRR........~~~~~~~~~~~~
+~~~~~~~~~~RRRRRRRRooooRRRRRR...........~~~~~~~~~~~
+~RRRRRRRRRRRRRRooooRRRRRRRR.............~~x~~~~~~~
+RRRRRRRRRRRoooooRRRRRRRRR...........#...~~~~~~~~~~
+RRRRRRRoooooRRRRRRRRRR........._.........~~~~~~~~~
+RRR+ooooRRRRRRRRRRR.................R.....~~~~~~~~
+RRRRRRRRRRRRRRRR..........................~~~~~~~~
+RRRRRRRRRRRRR.............................~~~~~~~~
+RRRRRRRRRR..........#........#.............~~~~~~~
+R~~~~~~~...................................~~~~~~~
+~~~~~~~~......._.......................#...~~~~~~~
+~~~~~~~~............R......................~~~~~~~
+~~~~~~~~.................?.................~~~~~~~
+~~~~x~~..................L.......R...._.....~~~~~~
+~~~~~~~~...................................~TTTTTT
+~~~~~~~~...............................TTTTTTTTTTT
+~~~~~~~~..........................TTTTTTTTT.TTTTTT
+~~~~~~~~.................#......TTTTT.TT.TT.TT.T+T
+~~~~~~~~......................TT..TTT.TT.T.TT.o.TT
+~~~~~~~~~.......#...........TTT.TT.TT.T.T.TTTT.TTT
+~~~~~~~~~.................TTTT.TT.TT.T.TTTTTTTTTTT
+~~~~~~~~~...............TTTTTT.T.TTT..TTTTTT~~~~~~
+~~~~~~~~~~............TTTTT.TT..TTTTTTT..~~~~~~~~~
+~~~~~~~x~~.........TTTTTTT.TTTTTT.......~~~~~~~~~~
+~~~~~~~~~~~........TTTTT.T.TTTTT.....o..~~~~~~~~~~
+~~~~~~~~~~~~......TT.TT..T.TTT.&amp;&amp;&amp;..o..~~~~~~~~~~~
+~~~~~~~~~~~~~...TTTT.T.TT.TT..&amp;!..&amp;...~~~~~~~~~~~~
+~~~~~~~~~~~~~~.TT.TT..TTTT...&amp;.!!.&amp;..~~~~~~~~~~~~~
+~~~~~~~~~~~~~~TT.o.T.TTT......&amp;.&amp;&amp;.~~~~~~~~~~~~~~~
+~~~~~~~~~~~~~TTTT.o..T...o.....&amp;..~~~~~~~~~~~~~~~~
+~~~~~~~~~~~~TTT+TT.TTT......o..~~~~~~~~~~~~~~~~~~~
+~~~~~~~~~~~~TTTTTTTT~~~~~.~~~~~~~~~~~~~~~~~~~~~~~~
+~~~~~~~~~~~TTTTTTTT~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~
+~~~~~~~~~~~TT.TTTT~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~
+~~~~~~~~~~TT.*.TT~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~
+~~~~~~~~~~TTT.TTT~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~
+~~~~~~~~~TTTTTTT~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~
+~~~~~~~~~TTTTTTT~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~</t>
+  </si>
+  <si>
+    <t>Onboarding</t>
+  </si>
+  <si>
+    <t>❤️</t>
+  </si>
+  <si>
+    <t>Rocky Road</t>
+  </si>
+  <si>
+    <t>Ice cream not for sale</t>
+  </si>
+  <si>
+    <t>20 25
+.RR.....RR...............
+RR.......RR...........+..
+R......._.R.........L....
+...+.......R.............
+........._.R.....T.......
+..~........R.............
+.~~........R........TT...
+......+..._R........T....
+R.........R..............
+RR.......RR..............
+.RR.....RR...._......T...
+...RRRRR............TT...
+............._......_....
+........_................
+...T..............RRRRR..
+..TT............RR.....RR
+...............RR.......R
+....+....T...._R....+....
+.........TT...R...~......
+..............R..........</t>
+  </si>
+  <si>
+    <t>Dark Forest</t>
+  </si>
+  <si>
+    <t>10 20
+.TTT.TT.T..T.TT.....
+..TT.T...T.T.....T.T
+..T.L?.....T.TT.T.TT
+T..TT....TT.T..TT..T
+.....T......xT...TT.
+T..........TT.+...T.
+..T..T.T..TT.......T
+TT...T....T.T.TT....
+TT..TT....TT....TT..
+TT.T...T.....T..T...</t>
+  </si>
+  <si>
+    <t>Sometimes, violence is the answer.</t>
+  </si>
+  <si>
+    <t>Timberland</t>
+  </si>
+  <si>
+    <t>Chop chop!</t>
+  </si>
+  <si>
+    <t>To The Other Side</t>
+  </si>
+  <si>
+    <t>So close, yet so far?</t>
+  </si>
+  <si>
+    <t>Beached Ship</t>
+  </si>
+  <si>
+    <t>This boat got stuck on ice...</t>
+  </si>
+  <si>
+    <t>🔴</t>
+  </si>
+  <si>
+    <t>Welcome to Shroom Raider!</t>
+  </si>
+  <si>
+    <t>25 25
+TTTTTT...+...TTTTTTTTTTT.
+TTTTTT.......TTTTT.TTTTT.
+TT.TTTTTTTTTTTTTT...TTTT.
+TTTTTTTTTTTTTTTT..+..TTT.
+TTTTTTTTTTTTTTTTT...TTTTT
+TTTTTTTTTT.TTTTTTT.TTTTTT
+..TTTTT......TTTTTTTTTTTT
+..TTTT_..R....TTTTTTTTT..
++.TTTT..R.RR...TTTTTTT.x.
+..TTTT..R.L.R..TTTTTT....
+..TTT..R.*+.R....TT...+..
+T_TTTT..R..x.R.TTTTTT....
+TTTTTT..RR_RR..TTTTTT.x..
+TTTTTT....R....TTTTTTTT..
+TTTTTTT.......TTTTTTTTTTT
+TTTTTTTTTT.TTTTTTTTTTTTTT
+TTT.TTTTTTTTTTTTTTTTTTTTT
+TTT..TTTTTTTTTTTTTTT.TTTT
+TTT...TTTTTTTTTTTT.....TT
+TTTTTTTT..._..TTTT.....TT
+TTTTTTTTT...._TTT...+...T
+T.TTTTTTT.....TTTT.....TT
+..TTT.TTT..+..TTTT.....TT
+..TTTTTTT.....TTTTTT.TTTT
+..TTTTTTT......TTTTTTTTTT</t>
+  </si>
+  <si>
+    <t>15 29
+........._..o...o......TTT...
+....._......oo.oo....._.TTT+.
+............ooooo.......+TTT.
+.....+......ooooo........TTTT
+.............ooo...........TT
+ooooooooooo.ooooo.ooooooooooo
+.ooooo.ooooooooooooooo.ooooo.
+..ooo.+.ooooooLoooooo.+.ooo..
+.ooooo.ooooooooooooooo.ooooo.
+ooooooooooo.ooooo.ooooooooooo
+TTT..........ooo.............
+.TTT........ooooo........._..
+..TTT.......ooooo......._....
+.+.TTT......oo.oo.........*..
+...TTT......o...o............</t>
+  </si>
+  <si>
+    <t>25 30
+......~~~~~~~~~~~~~~..........
+......~~~~~~~~~~~~~.......R...
+.....~~~~~~~~~~~~~~....R......
+..R..~~~~~~~~~~~~.........T+..
+......~~~~~~~~~~.......R...T..
+.+....~~~~~~~~~~~........._...
+.......~~~~~~~~~~~~.....R.....
+..._.....~~~~~~~~~~~....R.....
+......R....~~~~~~~~~~......TT.
+..T.........~~~~~~~~~......T..
+.............~~~~~~~~~.....~..
+.............~~~~~~~~.....~R~.
+.....R......~~~~~~~~~...~~RLR~
+...........~~~~~~~~.......~R~.
+..._.....~~~~~~~~~~...R....~..
+.......~~~~~~~~~~~..........R.
+......~~~~~~~~~~~.......R.....
+._....~~~~~~~~~~~....+........
+...T.~~~~~~~~~~..........R....
+..T..~~~~~~~~~~~~.............
+......~~~~~~~~~~~~...._.TT....
+......~~~~~~~~~~~~~~~~........
+..R....~~~~~~~~~~~~~~~~~...R..
+..__..~~~~~~~~~~~~~~~~~~......
+......~~~~~~~~~~~~~~~~~~~.....</t>
+  </si>
+  <si>
+    <t>27 11
+~~~~~~~~~~~
+~~~~~~~~~~~
+~#~TTTTT~#~
+~#TT.o.TT~#
+#TT..#..TT#
+.T.....~~T~
+TT..T.T~.TT
+T.x.T+T...T
+T...T~T.x.T
+TTTTT~TTTTT
+#~........T
+T..#...R..#
+T...~~~...T
+T#...T....T
+TT..~~~..TT
+.TT.....TT.
+..T..~..T..
+.#TT...TT..
+...T...T.#.
+~~.TT.TT.~.
+.~..T#T..__
+.#~....~~#.
+..~..L.~...
+.~~.....#..
+#~..R.R._..
+.~.RR~RR.~.
+_..RR+RR...</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -557,6 +835,24 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="7"/>
       <color theme="1"/>
       <name val="Courier New"/>
       <family val="3"/>
@@ -582,7 +878,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -604,6 +900,30 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -885,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1E384E5-DA51-499D-8241-92ECB4AE2D20}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.1328125" style="6"/>
@@ -938,6 +1258,17 @@
         <v>54</v>
       </c>
     </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" s="6">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>88</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -946,7 +1277,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
@@ -1249,7 +1580,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="384.75" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" ht="384.75" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -1263,7 +1594,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="409.5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1275,6 +1606,39 @@
       </c>
       <c r="E18" s="1" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="399" x14ac:dyDescent="0.45">
+      <c r="A19" s="1">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="409.6" x14ac:dyDescent="0.45">
+      <c r="A20" s="8">
+        <v>19</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" s="10"/>
+      <c r="E20" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1863,4 +2227,235 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFDB5384-A156-43AF-A2B8-6A3ECF7624E8}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="5" max="5" width="48.1328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="29.25" x14ac:dyDescent="0.5">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="171" x14ac:dyDescent="0.45">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+    </row>
+    <row r="3" spans="1:7" ht="196.9" x14ac:dyDescent="0.45">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+    </row>
+    <row r="4" spans="1:7" ht="103.15" x14ac:dyDescent="0.45">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="F4" s="15">
+        <v>3</v>
+      </c>
+      <c r="G4" s="14"/>
+    </row>
+    <row r="5" spans="1:7" ht="243.75" x14ac:dyDescent="0.45">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+    </row>
+    <row r="6" spans="1:7" ht="253.15" x14ac:dyDescent="0.45">
+      <c r="A6" s="9">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" s="14"/>
+      <c r="G6" s="15"/>
+    </row>
+    <row r="7" spans="1:7" ht="409.6" x14ac:dyDescent="0.45">
+      <c r="A7" s="9">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+    </row>
+    <row r="8" spans="1:7" ht="150" x14ac:dyDescent="0.45">
+      <c r="A8" s="9">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+    </row>
+    <row r="9" spans="1:7" ht="243.75" x14ac:dyDescent="0.45">
+      <c r="A9" s="9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+    </row>
+    <row r="10" spans="1:7" ht="262.5" x14ac:dyDescent="0.45">
+      <c r="A10" s="9">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+    </row>
+    <row r="11" spans="1:7" ht="409.6" x14ac:dyDescent="0.45">
+      <c r="A11" s="8">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="F11" s="10"/>
+      <c r="G11" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add Log sound and other fixes
</commit_message>
<xml_diff>
--- a/Bonus/Levels/levels_list.xlsx
+++ b/Bonus/Levels/levels_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Bonus\Levels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53EA744B-7DBF-46D8-BDE6-A4C707D9282E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44CE5FDE-4D27-47F5-B468-B777398A093D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="95">
   <si>
     <t>ID</t>
   </si>
@@ -812,6 +812,17 @@
 #~..R.R._..
 .~.RR~RR.~.
 _..RR+RR...</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>5 20
+.................~~~
+....T...........~~~~
+..+....T.ox.L..~~~~~
+.....T.........~~~~~
+................~~~~</t>
   </si>
 </sst>
 </file>
@@ -2231,7 +2242,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFDB5384-A156-43AF-A2B8-6A3ECF7624E8}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="5" max="5" width="48.1328125" customWidth="1"/>
@@ -2260,7 +2271,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="171" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" ht="185.25" x14ac:dyDescent="0.45">
       <c r="A2" s="9">
         <v>1</v>
       </c>
@@ -2452,6 +2463,23 @@
       <c r="F11" s="10"/>
       <c r="G11" s="12" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="56.25" x14ac:dyDescent="0.45">
+      <c r="A12" s="9">
+        <v>11</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>